<commit_message>
docs: reconcile native extraction follow-up with sanitized main roadmap
</commit_message>
<xml_diff>
--- a/gestaltdb_reasoning_feature_tracker.xlsx
+++ b/gestaltdb_reasoning_feature_tracker.xlsx
@@ -12,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Register'!$A$1:$N$137</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dashboard'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roadmap'!$A$1:$F$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roadmap'!$A$1:$F$36</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -619,12 +619,12 @@
       </c>
       <c r="M2" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -687,12 +687,12 @@
       </c>
       <c r="M3" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N3" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -755,12 +755,12 @@
       </c>
       <c r="M4" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -823,12 +823,12 @@
       </c>
       <c r="M5" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -891,12 +891,12 @@
       </c>
       <c r="M6" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1095,12 @@
       </c>
       <c r="M9" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1163,12 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="M11" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1299,12 +1299,12 @@
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1435,12 @@
       </c>
       <c r="M14" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1503,12 +1503,12 @@
       </c>
       <c r="M15" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1639,12 +1639,12 @@
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1707,12 +1707,12 @@
       </c>
       <c r="M18" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1775,12 +1775,12 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1843,12 +1843,12 @@
       </c>
       <c r="M20" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1911,12 +1911,12 @@
       </c>
       <c r="M21" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2047,12 +2047,12 @@
       </c>
       <c r="M23" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2115,12 +2115,12 @@
       </c>
       <c r="M24" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="M26" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2319,12 @@
       </c>
       <c r="M27" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2387,12 +2387,12 @@
       </c>
       <c r="M28" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="M29" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2523,12 +2523,12 @@
       </c>
       <c r="M30" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="M31" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2659,12 +2659,12 @@
       </c>
       <c r="M32" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2727,12 +2727,12 @@
       </c>
       <c r="M33" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2795,12 +2795,12 @@
       </c>
       <c r="M34" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2863,12 +2863,12 @@
       </c>
       <c r="M35" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2931,12 +2931,12 @@
       </c>
       <c r="M36" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="M37" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3067,12 +3067,12 @@
       </c>
       <c r="M38" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3135,12 +3135,12 @@
       </c>
       <c r="M39" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3203,12 +3203,12 @@
       </c>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="M41" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3339,12 +3339,12 @@
       </c>
       <c r="M42" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3407,12 +3407,12 @@
       </c>
       <c r="M43" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3475,12 +3475,12 @@
       </c>
       <c r="M44" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3543,12 +3543,12 @@
       </c>
       <c r="M45" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3611,12 +3611,12 @@
       </c>
       <c r="M46" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3679,12 +3679,12 @@
       </c>
       <c r="M47" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3747,12 +3747,12 @@
       </c>
       <c r="M48" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3815,12 +3815,12 @@
       </c>
       <c r="M49" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3883,12 +3883,12 @@
       </c>
       <c r="M50" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -3951,12 +3951,12 @@
       </c>
       <c r="M51" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4087,12 +4087,12 @@
       </c>
       <c r="M53" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="M54" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4223,12 +4223,12 @@
       </c>
       <c r="M55" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4291,12 @@
       </c>
       <c r="M56" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4359,12 +4359,12 @@
       </c>
       <c r="M57" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4427,12 +4427,12 @@
       </c>
       <c r="M58" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4495,12 +4495,12 @@
       </c>
       <c r="M59" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4563,12 +4563,12 @@
       </c>
       <c r="M60" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4631,12 +4631,12 @@
       </c>
       <c r="M61" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4699,12 +4699,12 @@
       </c>
       <c r="M62" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4767,12 +4767,12 @@
       </c>
       <c r="M63" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4835,12 +4835,12 @@
       </c>
       <c r="M64" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4903,12 +4903,12 @@
       </c>
       <c r="M65" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -4971,12 +4971,12 @@
       </c>
       <c r="M66" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5039,12 @@
       </c>
       <c r="M67" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5107,12 +5107,12 @@
       </c>
       <c r="M68" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5175,12 +5175,12 @@
       </c>
       <c r="M69" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5243,12 +5243,12 @@
       </c>
       <c r="M70" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5311,12 @@
       </c>
       <c r="M71" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5379,12 +5379,12 @@
       </c>
       <c r="M72" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5447,12 +5447,12 @@
       </c>
       <c r="M73" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="M74" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5583,12 +5583,12 @@
       </c>
       <c r="M75" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5651,12 +5651,12 @@
       </c>
       <c r="M76" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5719,12 +5719,12 @@
       </c>
       <c r="M77" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5787,12 +5787,12 @@
       </c>
       <c r="M78" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5855,12 +5855,12 @@
       </c>
       <c r="M79" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5923,12 +5923,12 @@
       </c>
       <c r="M80" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -5991,12 +5991,12 @@
       </c>
       <c r="M81" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6059,12 +6059,12 @@
       </c>
       <c r="M82" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6127,12 +6127,12 @@
       </c>
       <c r="M83" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6195,12 +6195,12 @@
       </c>
       <c r="M84" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6263,12 @@
       </c>
       <c r="M85" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6331,12 +6331,12 @@
       </c>
       <c r="M86" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6399,12 +6399,12 @@
       </c>
       <c r="M87" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6467,12 +6467,12 @@
       </c>
       <c r="M88" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6535,12 +6535,12 @@
       </c>
       <c r="M89" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6603,12 +6603,12 @@
       </c>
       <c r="M90" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6671,12 +6671,12 @@
       </c>
       <c r="M91" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6739,12 +6739,12 @@
       </c>
       <c r="M92" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6807,12 @@
       </c>
       <c r="M93" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6875,12 +6875,12 @@
       </c>
       <c r="M94" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -6943,12 +6943,12 @@
       </c>
       <c r="M95" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7011,12 +7011,12 @@
       </c>
       <c r="M96" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7079,12 +7079,12 @@
       </c>
       <c r="M97" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7147,12 +7147,12 @@
       </c>
       <c r="M98" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7215,12 +7215,12 @@
       </c>
       <c r="M99" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N99" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7283,12 @@
       </c>
       <c r="M100" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N100" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7351,12 +7351,12 @@
       </c>
       <c r="M101" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N101" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7419,12 +7419,12 @@
       </c>
       <c r="M102" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N102" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7487,12 +7487,12 @@
       </c>
       <c r="M103" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N103" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7555,12 +7555,12 @@
       </c>
       <c r="M104" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N104" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7623,12 +7623,12 @@
       </c>
       <c r="M105" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N105" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7691,12 +7691,12 @@
       </c>
       <c r="M106" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N106" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7759,12 +7759,12 @@
       </c>
       <c r="M107" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7827,12 @@
       </c>
       <c r="M108" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N108" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7895,12 +7895,12 @@
       </c>
       <c r="M109" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -7963,12 +7963,12 @@
       </c>
       <c r="M110" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8031,12 +8031,12 @@
       </c>
       <c r="M111" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8099,12 +8099,12 @@
       </c>
       <c r="M112" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8167,12 +8167,12 @@
       </c>
       <c r="M113" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N113" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8235,12 +8235,12 @@
       </c>
       <c r="M114" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N114" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8303,12 +8303,12 @@
       </c>
       <c r="M115" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N115" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8371,12 +8371,12 @@
       </c>
       <c r="M116" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N116" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8439,12 +8439,12 @@
       </c>
       <c r="M117" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8507,12 +8507,12 @@
       </c>
       <c r="M118" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8575,12 +8575,12 @@
       </c>
       <c r="M119" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8643,12 +8643,12 @@
       </c>
       <c r="M120" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8711,12 +8711,12 @@
       </c>
       <c r="M121" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N121" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8779,12 +8779,12 @@
       </c>
       <c r="M122" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8847,12 +8847,12 @@
       </c>
       <c r="M123" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N123" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8915,12 +8915,12 @@
       </c>
       <c r="M124" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N124" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -8983,12 +8983,12 @@
       </c>
       <c r="M125" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9051,12 +9051,12 @@
       </c>
       <c r="M126" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9119,12 +9119,12 @@
       </c>
       <c r="M127" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N127" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9187,12 +9187,12 @@
       </c>
       <c r="M128" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N128" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9255,12 +9255,12 @@
       </c>
       <c r="M129" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N129" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9323,12 +9323,12 @@
       </c>
       <c r="M130" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N130" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9391,12 +9391,12 @@
       </c>
       <c r="M131" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N131" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9459,12 +9459,12 @@
       </c>
       <c r="M132" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N132" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9527,12 +9527,12 @@
       </c>
       <c r="M133" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N133" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9595,12 +9595,12 @@
       </c>
       <c r="M134" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N134" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9663,12 +9663,12 @@
       </c>
       <c r="M135" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N135" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9731,12 +9731,12 @@
       </c>
       <c r="M136" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N136" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9799,12 +9799,12 @@
       </c>
       <c r="M137" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="N137" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -9985,7 +9985,7 @@
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T11:27:42Z</t>
+          <t>2026-11-01T13:00:35Z</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>3403530adf186cf79d6426829d3be8bf8898f6f3</t>
+          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>#194: Open; implemented source, pending measurement; #124: Open proposal; design-gated; #128: Open composition proposal; #388: Open, partially delivered; #410: Open, partially delivered; #273: Open documentation track; #409: Open application proposal</t>
+          <t>#194: Open; implemented source on main; measurement/decision in unmerged #450; #451: Open technical debt; not remediated; #124: Open proposal; design-gated; #128: Open composition proposal; #388: Open, partially delivered; #410: Open, partially delivered; #273: Open documentation track; #409: Open application proposal</t>
         </is>
       </c>
     </row>
@@ -10207,7 +10207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11122,17 +11122,17 @@
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Open; implemented source, pending measurement</t>
+          <t>Open; implemented source on main; measurement/decision in unmerged #450</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Benchmark actual `PinnedNativeLocatorClaimSource` with named historical/selective and nonselective inputs, complete authentication/point materialization, exact evidence/closure parity, versions, time/RSS and explicit adoption decision. Do not substitute benchmark-only locator, raw KV or full-record native results. Optional, not a #156 blocker.</t>
+          <t>PR #450 preserves 18/18 exact fact/version-ID parity observations at 100K sparse history, including selective/nonselective reads and full authentication/materialization costs, versions and time/RSS. Decision: defer automatic native adoption. Complete integration/review; no rule-closure, repeated-performance or OS-cold claim. Do not substitute raw/assertion-only/full-record modes. Optional, not a #156 blocker.</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E29" s="19" t="n"/>
@@ -11145,22 +11145,22 @@
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#451</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Open proposal; design-gated</t>
+          <t>Open technical debt; not remediated</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Choose probabilistic, fuzzy **or** importance semantics; prove combination, retraction, convergence and provenance with independent tests and a named user scenario. No silent confidence multiplication.</t>
+          <t>Resolve dense-history supersession/commit validation and native locator read amplification without weakening authentication. Dense 100K construction timed out at 900 s before extraction; sparse-history success is different evidence. Instrument/batch verified target resolution, bound redundant catalog/history work and remeasure isolated repeated time/RSS. Native adoption remains deferred.</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E30" s="19" t="n"/>
@@ -11173,22 +11173,22 @@
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>#128</t>
+          <t>#124</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Open composition proposal</t>
+          <t>Open proposal; design-gated</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Model/task/version provenance, source/world/assertion policy, bounded iterations and leakage controls. Weighted feedback depends on #124; a small deterministic loop need not. Audit export #126 is delivered.</t>
+          <t>Choose probabilistic, fuzzy **or** importance semantics; prove combination, retraction, convergence and provenance with independent tests and a named user scenario. No silent confidence multiplication.</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E31" s="19" t="n"/>
@@ -11201,22 +11201,22 @@
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>#388</t>
+          <t>#128</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>Open, partially delivered</t>
+          <t>Open composition proposal</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Finish concrete facade/consumer coupling: legacy adjacency/BFS, update composition, key/serializer helpers and query/viz/transaction/snapshot/lifecycle integration. Services already exist; require standalone boundary/compatibility tests, not a facade line-count goal.</t>
+          <t>Model/task/version provenance, source/world/assertion policy, bounded iterations and leakage controls. Weighted feedback depends on #124; a small deterministic loop need not. Audit export #126 is delivered.</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E32" s="19" t="n"/>
@@ -11229,7 +11229,7 @@
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>#410</t>
+          <t>#388</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -11239,12 +11239,12 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Remaining diagnostics, read-view/facade and optional adapter contracts, normalized construction inputs and installed consumer checks. `py.typed` and scoped strict ratchets already ship. Old diagnostic totals are not current runtime bug counts.</t>
+          <t>Finish concrete facade/consumer coupling: legacy adjacency/BFS, update composition, key/serializer helpers and query/viz/transaction/snapshot/lifecycle integration. Services already exist; require standalone boundary/compatibility tests, not a facade line-count goal.</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E33" s="19" t="n"/>
@@ -11257,22 +11257,22 @@
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>#273</t>
+          <t>#410</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>Open documentation track</t>
+          <t>Open, partially delivered</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Complete/reconcile tutorial coverage and publish from its separate branch; old gap lists need current fragments. Not a missing core engine.</t>
+          <t>Remaining diagnostics, read-view/facade and optional adapter contracts, normalized construction inputs and installed consumer checks. `py.typed` and scoped strict ratchets already ship. Old diagnostic totals are not current runtime bug counts.</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E34" s="19" t="n"/>
@@ -11285,22 +11285,22 @@
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>#409</t>
+          <t>#273</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>Open application proposal</t>
+          <t>Open documentation track</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>CDM schema impact, collateral/lifecycle/temporal-ML scenarios with explicit expected results and data/version policies. No automatic CDM/Rune translation or financial-calculation semantics implied.</t>
+          <t>Complete/reconcile tutorial coverage and publish from its separate branch; old gap lists need current fragments. Not a missing core engine.</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T11:27:42Z</t>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
         </is>
       </c>
       <c r="E35" s="19" t="n"/>
@@ -11310,8 +11310,36 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>#409</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Open application proposal</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>CDM schema impact, collateral/lifecycle/temporal-ML scenarios with explicit expected results and data/version policies. No automatic CDM/Rune translation or financial-calculation semantics implied.</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Reviewed 2026-11-01T13:00:35Z</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>See remaining scope</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F35"/>
+  <autoFilter ref="A1:F36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
benchmarks: record HSA acceptance pilot and reconcile defer boundaries
</commit_message>
<xml_diff>
--- a/gestaltdb_reasoning_feature_tracker.xlsx
+++ b/gestaltdb_reasoning_feature_tracker.xlsx
@@ -619,12 +619,12 @@
       </c>
       <c r="M2" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -687,12 +687,12 @@
       </c>
       <c r="M3" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N3" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -755,12 +755,12 @@
       </c>
       <c r="M4" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -823,12 +823,12 @@
       </c>
       <c r="M5" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -891,12 +891,12 @@
       </c>
       <c r="M6" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1095,12 @@
       </c>
       <c r="M9" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1163,12 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="M11" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1299,12 +1299,12 @@
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1435,12 @@
       </c>
       <c r="M14" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1503,12 +1503,12 @@
       </c>
       <c r="M15" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1639,12 +1639,12 @@
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1707,12 +1707,12 @@
       </c>
       <c r="M18" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1775,12 +1775,12 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1843,12 +1843,12 @@
       </c>
       <c r="M20" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1911,12 +1911,12 @@
       </c>
       <c r="M21" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="M22" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2047,12 +2047,12 @@
       </c>
       <c r="M23" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2115,12 +2115,12 @@
       </c>
       <c r="M24" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="M26" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2319,12 +2319,12 @@
       </c>
       <c r="M27" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2387,12 +2387,12 @@
       </c>
       <c r="M28" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="M29" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2523,12 +2523,12 @@
       </c>
       <c r="M30" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="M31" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2659,12 +2659,12 @@
       </c>
       <c r="M32" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2727,12 +2727,12 @@
       </c>
       <c r="M33" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2795,12 +2795,12 @@
       </c>
       <c r="M34" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2863,12 +2863,12 @@
       </c>
       <c r="M35" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2931,12 +2931,12 @@
       </c>
       <c r="M36" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="M37" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3067,12 +3067,12 @@
       </c>
       <c r="M38" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3135,12 +3135,12 @@
       </c>
       <c r="M39" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3203,12 +3203,12 @@
       </c>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="M41" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3339,12 +3339,12 @@
       </c>
       <c r="M42" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3407,12 +3407,12 @@
       </c>
       <c r="M43" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3475,12 +3475,12 @@
       </c>
       <c r="M44" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3543,12 +3543,12 @@
       </c>
       <c r="M45" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3611,12 +3611,12 @@
       </c>
       <c r="M46" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3679,12 +3679,12 @@
       </c>
       <c r="M47" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3747,12 +3747,12 @@
       </c>
       <c r="M48" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3815,12 +3815,12 @@
       </c>
       <c r="M49" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3883,12 +3883,12 @@
       </c>
       <c r="M50" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -3951,12 +3951,12 @@
       </c>
       <c r="M51" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4087,12 +4087,12 @@
       </c>
       <c r="M53" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="M54" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4223,12 +4223,12 @@
       </c>
       <c r="M55" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4291,12 @@
       </c>
       <c r="M56" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4359,12 +4359,12 @@
       </c>
       <c r="M57" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4427,12 +4427,12 @@
       </c>
       <c r="M58" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4495,12 +4495,12 @@
       </c>
       <c r="M59" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4563,12 +4563,12 @@
       </c>
       <c r="M60" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4631,12 +4631,12 @@
       </c>
       <c r="M61" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4699,12 +4699,12 @@
       </c>
       <c r="M62" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4767,12 +4767,12 @@
       </c>
       <c r="M63" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4835,12 +4835,12 @@
       </c>
       <c r="M64" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4903,12 +4903,12 @@
       </c>
       <c r="M65" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -4971,12 +4971,12 @@
       </c>
       <c r="M66" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5039,12 +5039,12 @@
       </c>
       <c r="M67" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5107,12 +5107,12 @@
       </c>
       <c r="M68" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5175,12 +5175,12 @@
       </c>
       <c r="M69" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5243,12 +5243,12 @@
       </c>
       <c r="M70" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5311,12 @@
       </c>
       <c r="M71" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5379,12 +5379,12 @@
       </c>
       <c r="M72" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5447,12 +5447,12 @@
       </c>
       <c r="M73" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="M74" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5583,12 +5583,12 @@
       </c>
       <c r="M75" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5651,12 +5651,12 @@
       </c>
       <c r="M76" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5719,12 +5719,12 @@
       </c>
       <c r="M77" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5787,12 +5787,12 @@
       </c>
       <c r="M78" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5855,12 +5855,12 @@
       </c>
       <c r="M79" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5923,12 +5923,12 @@
       </c>
       <c r="M80" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -5991,12 +5991,12 @@
       </c>
       <c r="M81" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6059,12 +6059,12 @@
       </c>
       <c r="M82" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6127,12 +6127,12 @@
       </c>
       <c r="M83" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6195,12 +6195,12 @@
       </c>
       <c r="M84" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6263,12 @@
       </c>
       <c r="M85" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6331,12 +6331,12 @@
       </c>
       <c r="M86" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6399,12 +6399,12 @@
       </c>
       <c r="M87" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6467,12 +6467,12 @@
       </c>
       <c r="M88" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6535,12 +6535,12 @@
       </c>
       <c r="M89" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6603,12 +6603,12 @@
       </c>
       <c r="M90" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6671,12 +6671,12 @@
       </c>
       <c r="M91" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6739,12 +6739,12 @@
       </c>
       <c r="M92" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6807,12 @@
       </c>
       <c r="M93" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6875,12 +6875,12 @@
       </c>
       <c r="M94" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -6943,12 +6943,12 @@
       </c>
       <c r="M95" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7011,12 +7011,12 @@
       </c>
       <c r="M96" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7079,12 +7079,12 @@
       </c>
       <c r="M97" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7147,12 +7147,12 @@
       </c>
       <c r="M98" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7215,12 +7215,12 @@
       </c>
       <c r="M99" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N99" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7283,12 @@
       </c>
       <c r="M100" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N100" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7351,12 +7351,12 @@
       </c>
       <c r="M101" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N101" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7419,12 +7419,12 @@
       </c>
       <c r="M102" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N102" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7487,12 +7487,12 @@
       </c>
       <c r="M103" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N103" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7555,12 +7555,12 @@
       </c>
       <c r="M104" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N104" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7623,12 +7623,12 @@
       </c>
       <c r="M105" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N105" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7691,12 +7691,12 @@
       </c>
       <c r="M106" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N106" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7759,12 +7759,12 @@
       </c>
       <c r="M107" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7827,12 +7827,12 @@
       </c>
       <c r="M108" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N108" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7895,12 +7895,12 @@
       </c>
       <c r="M109" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -7963,12 +7963,12 @@
       </c>
       <c r="M110" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8031,12 +8031,12 @@
       </c>
       <c r="M111" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8099,12 +8099,12 @@
       </c>
       <c r="M112" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8167,12 +8167,12 @@
       </c>
       <c r="M113" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N113" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8235,12 +8235,12 @@
       </c>
       <c r="M114" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N114" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8303,12 +8303,12 @@
       </c>
       <c r="M115" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N115" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8371,12 +8371,12 @@
       </c>
       <c r="M116" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N116" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8439,12 +8439,12 @@
       </c>
       <c r="M117" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8507,12 +8507,12 @@
       </c>
       <c r="M118" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8575,12 +8575,12 @@
       </c>
       <c r="M119" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8643,12 +8643,12 @@
       </c>
       <c r="M120" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8711,12 +8711,12 @@
       </c>
       <c r="M121" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N121" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8779,12 +8779,12 @@
       </c>
       <c r="M122" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8847,12 +8847,12 @@
       </c>
       <c r="M123" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N123" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8915,12 +8915,12 @@
       </c>
       <c r="M124" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N124" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -8983,12 +8983,12 @@
       </c>
       <c r="M125" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9051,12 +9051,12 @@
       </c>
       <c r="M126" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9119,12 +9119,12 @@
       </c>
       <c r="M127" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N127" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9187,12 +9187,12 @@
       </c>
       <c r="M128" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N128" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9255,12 +9255,12 @@
       </c>
       <c r="M129" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N129" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9323,12 +9323,12 @@
       </c>
       <c r="M130" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N130" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9391,12 +9391,12 @@
       </c>
       <c r="M131" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N131" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9459,12 +9459,12 @@
       </c>
       <c r="M132" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N132" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9527,12 +9527,12 @@
       </c>
       <c r="M133" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N133" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9595,12 +9595,12 @@
       </c>
       <c r="M134" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N134" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9663,12 +9663,12 @@
       </c>
       <c r="M135" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N135" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9731,12 +9731,12 @@
       </c>
       <c r="M136" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N136" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9799,12 +9799,12 @@
       </c>
       <c r="M137" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="N137" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -9985,7 +9985,7 @@
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>2026-11-01T13:00:35Z</t>
+          <t>2026-11-01T23:07:18Z</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>7f288085fc01ecd2fac66def9d3c29981054af26</t>
+          <t>dcc90e2b3c21875045f3760bcedd3a234cb79e42</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>#194: Open; implemented source on main; measurement/decision in unmerged #450; #451: Open technical debt; not remediated; #124: Open proposal; design-gated; #128: Open composition proposal; #388: Open, partially delivered; #410: Open, partially delivered; #273: Open documentation track; #409: Open application proposal</t>
+          <t>#194: Open; measurements/defer decision merged in #450; #451: Open technical debt; partial HSA work on hsa-dev; #124: Open proposal; design-gated; #128: Open composition proposal; #388: Open, partially delivered; #410: Open, partially delivered; #273: Open documentation track; #409: Open application proposal</t>
         </is>
       </c>
     </row>
@@ -11122,17 +11122,17 @@
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Open; implemented source on main; measurement/decision in unmerged #450</t>
+          <t>Open; measurements/defer decision merged in #450</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>PR #450 preserves 18/18 exact fact/version-ID parity observations at 100K sparse history, including selective/nonselective reads and full authentication/materialization costs, versions and time/RSS. Decision: defer automatic native adoption. Complete integration/review; no rule-closure, repeated-performance or OS-cold claim. Do not substitute raw/assertion-only/full-record modes. Optional, not a #156 blocker.</t>
+          <t>Main now contains the actual-adapter harness and original 18/18 sparse-history 100K plus 36/36 diagnostic dense 10K parity observations. Preserve their original source/host/cache limitations; no raw/assertion-only/full-record substitution or native adoption. Closure reconciliation remains separate from optimization debt #451. Optional, not a #156 blocker.</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E29" s="19" t="n"/>
@@ -11150,17 +11150,17 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Open technical debt; not remediated</t>
+          <t>Open technical debt; partial HSA work on hsa-dev</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Resolve dense-history supersession/commit validation and native locator read amplification without weakening authentication. Dense 100K construction timed out at 900 s before extraction; sparse-history success is different evidence. Instrument/batch verified target resolution, bound redundant catalog/history work and remeasure isolated repeated time/RSS. Native adoption remains deferred.</t>
+          <t>HSA-02 is on main; HSA-03/HSA-04 remain on hsa-dev. HSA-06 pilot: dense 100K/134286-version construction passes the preserved 900s gate in 35.17s, with checked-point parity; 216 unprofiled alternating 1K reads pass own-baseline observed gates, but selective native latency/RSS fails the 1.25x ordinary goal. Larger/warm/sparse paired gates and rollout remain; native adoption and optional new-index HSA-05 stay deferred. See planning/reasoning-followthrough/hsa-06-pilot.md; no blanket performance or feature promotion.</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E30" s="19" t="n"/>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E31" s="19" t="n"/>
@@ -11216,7 +11216,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E32" s="19" t="n"/>
@@ -11244,7 +11244,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E33" s="19" t="n"/>
@@ -11272,7 +11272,7 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E34" s="19" t="n"/>
@@ -11300,7 +11300,7 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E35" s="19" t="n"/>
@@ -11328,7 +11328,7 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Reviewed 2026-11-01T13:00:35Z</t>
+          <t>Reviewed 2026-11-01T23:07:18Z</t>
         </is>
       </c>
       <c r="E36" s="19" t="n"/>

</xml_diff>